<commit_message>
Add detailed report fields, reports page, and updated export/upload
</commit_message>
<xml_diff>
--- a/public/apprehension_upload_template.xlsx
+++ b/public/apprehension_upload_template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t xml:space="preserve">CENRO Office</t>
   </si>
@@ -28,34 +28,61 @@
     <t xml:space="preserve">Year</t>
   </si>
   <si>
+    <t xml:space="preserve">Month</t>
+  </si>
+  <si>
     <t xml:space="preserve">Date of Apprehension</t>
   </si>
   <si>
     <t xml:space="preserve">Place of Apprehension</t>
   </si>
   <si>
+    <t xml:space="preserve">Apprehending Agency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claimant/Respondent</t>
+  </si>
+  <si>
     <t xml:space="preserve">Circumstances</t>
   </si>
   <si>
     <t xml:space="preserve">Custodian Location</t>
   </si>
   <si>
-    <t xml:space="preserve">Other Agencies Involved</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conveyance/Equipment</t>
+    <t xml:space="preserve">Other Agencies</t>
   </si>
   <si>
     <t xml:space="preserve">Remarks</t>
   </si>
   <si>
-    <t xml:space="preserve">Item Description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Volume (cu.m.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimated Value (PHP)</t>
+    <t xml:space="preserve">Item Qty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item Species</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item Forms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item Volume (BDFT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item Volume (cu.m.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item Value (PHP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conveyance Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conveyance Qty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipment Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipment Qty</t>
   </si>
   <si>
     <t xml:space="preserve">Instructions</t>
@@ -64,10 +91,16 @@
     <t xml:space="preserve">APARRI</t>
   </si>
   <si>
-    <t xml:space="preserve">Jan. 16, 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Burubur, Magapit, Lal-lo, Cagayan</t>
+    <t xml:space="preserve">September 21, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sta. Ana, Gattaran, Cagayan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PNP Gattaran</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alfredo B. Pavo</t>
   </si>
   <si>
     <t xml:space="preserve">No permit/transport documents</t>
@@ -76,37 +109,46 @@
     <t xml:space="preserve">CENRO Aparri compound</t>
   </si>
   <si>
-    <t xml:space="preserve">PNP Lal-lo</t>
-  </si>
-  <si>
     <t xml:space="preserve">For resolution</t>
   </si>
   <si>
-    <t xml:space="preserve">8 pcs. Narra flitches</t>
+    <t xml:space="preserve">7 &amp; 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gmelina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lumber &amp; Round logs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chainsaw with defaced serial number</t>
   </si>
   <si>
     <t xml:space="preserve">1. Do not edit the header row (row 1).</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Row 2 (yellow) is an example — delete it or overwrite it with real data.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. CENRO Office must be one of: APARRI, ALCALA, SOLANA, SANCHEZ MIRA, TUGUEGARAO, SUB OFFICE.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Year must be a 4-digit number.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. One row = one apprehension record with one item. For multiple items in one</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   apprehension, repeat the row with the same Date/Place and a different item.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. Volume and Estimated Value should be numbers only (no currency symbols or commas).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7. Leave a cell blank if not applicable — do not write 'N/A' or '-'.</t>
+    <t xml:space="preserve">2. Row 2 (yellow) is an example — delete or overwrite it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. CENRO Office: APARRI, ALCALA, SOLANA, SANCHEZ MIRA, TUGUEGARAO, or SUB OFFICE.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Month must be a number 1–12 (e.g. 9 for September).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. One row = one apprehension with one forest-product item.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   For multiple items, repeat the row with the same date/place.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Conveyance/Equipment columns are optional — leave blank if none.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. Numbers only in Qty/Volume/Value columns — no currency symbols or commas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8. Leave a cell blank if not applicable — do not write 'N/A' or '-'.</t>
   </si>
 </sst>
 </file>
@@ -496,24 +538,32 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:W10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="15" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="55"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -550,82 +600,133 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="B2" s="3" t="n">
         <v>2026</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>14</v>
+      <c r="C2" s="3" t="n">
+        <v>9</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H2" s="3"/>
+        <v>26</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>27</v>
+      </c>
       <c r="I2" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" s="3" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="L2" s="3" t="n">
-        <v>45000</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>21</v>
+        <v>28</v>
+      </c>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="O2" s="3" t="n">
+        <v>354.4</v>
+      </c>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3"/>
+      <c r="R2" s="3"/>
+      <c r="S2" s="3"/>
+      <c r="T2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="U2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="W2" s="4" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N3" s="4" t="s">
-        <v>22</v>
+      <c r="W3" s="4" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N4" s="4" t="s">
-        <v>23</v>
+      <c r="W4" s="4" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N5" s="4" t="s">
-        <v>24</v>
+      <c r="W5" s="4" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N6" s="4" t="s">
-        <v>25</v>
+      <c r="W6" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N7" s="4" t="s">
-        <v>26</v>
+      <c r="W7" s="4" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N8" s="4" t="s">
-        <v>27</v>
+      <c r="W8" s="4" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N9" s="4" t="s">
-        <v>28</v>
+      <c r="W9" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="W10" s="4" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Edit the upload template and fix missing CENRO word save to DB
</commit_message>
<xml_diff>
--- a/public/apprehension_upload_template.xlsx
+++ b/public/apprehension_upload_template.xlsx
@@ -12116,7 +12116,7 @@
   </sheetData>
   <dataValidations count="8">
     <dataValidation sqref="A2:A500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid office" error="Pick one of the listed CENRO offices." type="list">
-      <formula1>"APARRI,ALCALA,SOLANA,SANCHEZ MIRA,TUGUEGARAO,SUB OFFICE"</formula1>
+      <formula1>"CENRO APARRI,CENRO ALCALA,CENRO SOLANA,CENRO SANCHEZ MIRA,CENRO TUGUEGARAO,SUB OFFICE"</formula1>
     </dataValidation>
     <dataValidation sqref="B2:B500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid year" error="Enter a year like 2026." type="whole" operator="between">
       <formula1>2000</formula1>
@@ -12198,7 +12198,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Pick from the dropdown: APARRI, ALCALA, SOLANA, SANCHEZ MIRA, TUGUEGARAO, SUB OFFICE.</t>
+          <t>Pick from the dropdown: CENRO APARRI, CENRO ALCALA, CENRO SOLANA, CENRO SANCHEZ MIRA, CENRO TUGUEGARAO, SUB OFFICE.</t>
         </is>
       </c>
     </row>
@@ -12313,7 +12313,7 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>APARRI</t>
+          <t>CENRO APARRI</t>
         </is>
       </c>
     </row>

</xml_diff>